<commit_message>
Fix Ezra and Asher problem
</commit_message>
<xml_diff>
--- a/photos/pdf_files.xlsx
+++ b/photos/pdf_files.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\soder\Documents\GitHub\soderstrand\photos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C14AB4C2-C48A-4DCE-80D7-41019C001C58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58D4050A-438A-4C1D-9A73-E55DA932A035}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -112,9 +112,6 @@
     <t>2023-06-06_dickeyville _tail.pdf</t>
   </si>
   <si>
-    <t>2023-11-18 ezra_asher's_1st_birthday.pdf</t>
-  </si>
-  <si>
     <t>2024-05-02_house_of_prime_rib.pdf</t>
   </si>
   <si>
@@ -278,6 +275,9 @@
   </si>
   <si>
     <t>2026-06-24 Columbus Pride Parade Columbus OH</t>
+  </si>
+  <si>
+    <t>2023-11-18 ezra_ashers_1st_birthday.pdf</t>
   </si>
 </sst>
 </file>
@@ -670,7 +670,7 @@
         <v>20</v>
       </c>
       <c r="D2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E2" t="s">
         <v>5</v>
@@ -687,10 +687,10 @@
         <v>7</v>
       </c>
       <c r="D3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
@@ -704,7 +704,7 @@
         <v>3</v>
       </c>
       <c r="D4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E4" t="s">
         <v>6</v>
@@ -721,7 +721,7 @@
         <v>22</v>
       </c>
       <c r="D5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E5" t="s">
         <v>9</v>
@@ -738,7 +738,7 @@
         <v>8</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E6" t="s">
         <v>8</v>
@@ -755,7 +755,7 @@
         <v>12</v>
       </c>
       <c r="D7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E7" t="s">
         <v>7</v>
@@ -772,7 +772,7 @@
         <v>9</v>
       </c>
       <c r="D8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E8" t="s">
         <v>10</v>
@@ -789,7 +789,7 @@
         <v>27</v>
       </c>
       <c r="D9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E9" t="s">
         <v>11</v>
@@ -806,7 +806,7 @@
         <v>6</v>
       </c>
       <c r="D10" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E10" t="s">
         <v>12</v>
@@ -823,10 +823,10 @@
         <v>7</v>
       </c>
       <c r="D11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E11" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
@@ -840,7 +840,7 @@
         <v>8</v>
       </c>
       <c r="D12" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E12" t="s">
         <v>13</v>
@@ -857,7 +857,7 @@
         <v>8</v>
       </c>
       <c r="D13" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E13" t="s">
         <v>14</v>
@@ -874,7 +874,7 @@
         <v>9</v>
       </c>
       <c r="D14" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E14" t="s">
         <v>15</v>
@@ -891,7 +891,7 @@
         <v>10</v>
       </c>
       <c r="D15" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E15" t="s">
         <v>16</v>
@@ -908,7 +908,7 @@
         <v>10</v>
       </c>
       <c r="D16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E16" t="s">
         <v>17</v>
@@ -925,10 +925,10 @@
         <v>3</v>
       </c>
       <c r="D17" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E17" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
@@ -942,7 +942,7 @@
         <v>16</v>
       </c>
       <c r="D18" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E18" t="s">
         <v>18</v>
@@ -959,7 +959,7 @@
         <v>1</v>
       </c>
       <c r="D19" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E19" t="s">
         <v>23</v>
@@ -976,7 +976,7 @@
         <v>10</v>
       </c>
       <c r="D20" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E20" t="s">
         <v>19</v>
@@ -993,7 +993,7 @@
         <v>12</v>
       </c>
       <c r="D21" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E21" t="s">
         <v>20</v>
@@ -1010,7 +1010,7 @@
         <v>12</v>
       </c>
       <c r="D22" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E22" t="s">
         <v>21</v>
@@ -1027,7 +1027,7 @@
         <v>23</v>
       </c>
       <c r="D23" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E23" t="s">
         <v>22</v>
@@ -1044,7 +1044,7 @@
         <v>25</v>
       </c>
       <c r="D24" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E24" t="s">
         <v>24</v>
@@ -1061,7 +1061,7 @@
         <v>15</v>
       </c>
       <c r="D25" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E25" t="s">
         <v>25</v>
@@ -1078,7 +1078,7 @@
         <v>21</v>
       </c>
       <c r="D26" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E26" t="s">
         <v>26</v>
@@ -1095,7 +1095,7 @@
         <v>3</v>
       </c>
       <c r="D27" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E27" t="s">
         <v>27</v>
@@ -1112,7 +1112,7 @@
         <v>6</v>
       </c>
       <c r="D28" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E28" t="s">
         <v>28</v>
@@ -1129,10 +1129,10 @@
         <v>18</v>
       </c>
       <c r="D29" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E29" t="s">
-        <v>29</v>
+        <v>84</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
@@ -1146,10 +1146,10 @@
         <v>2</v>
       </c>
       <c r="D30" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E30" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.35">
@@ -1163,10 +1163,10 @@
         <v>2</v>
       </c>
       <c r="D31" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E31" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.35">
@@ -1180,10 +1180,10 @@
         <v>3</v>
       </c>
       <c r="D32" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E32" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.35">
@@ -1197,10 +1197,10 @@
         <v>7</v>
       </c>
       <c r="D33" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E33" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.35">
@@ -1214,10 +1214,10 @@
         <v>14</v>
       </c>
       <c r="D34" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E34" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.35">
@@ -1231,10 +1231,10 @@
         <v>24</v>
       </c>
       <c r="D35" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E35" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.35">
@@ -1248,10 +1248,10 @@
         <v>11</v>
       </c>
       <c r="D36" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E36" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.35">
@@ -1265,10 +1265,10 @@
         <v>22</v>
       </c>
       <c r="D37" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E37" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.35">
@@ -1282,10 +1282,10 @@
         <v>14</v>
       </c>
       <c r="D38" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E38" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.35">
@@ -1299,10 +1299,10 @@
         <v>8</v>
       </c>
       <c r="D39" t="s">
+        <v>80</v>
+      </c>
+      <c r="E39" t="s">
         <v>81</v>
-      </c>
-      <c r="E39" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.35">
@@ -1316,10 +1316,10 @@
         <v>11</v>
       </c>
       <c r="D40" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E40" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.35">
@@ -1333,10 +1333,10 @@
         <v>24</v>
       </c>
       <c r="D41" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E41" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add 2500 Pickwick Photos
</commit_message>
<xml_diff>
--- a/photos/pdf_files.xlsx
+++ b/photos/pdf_files.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\soder\Documents\GitHub\soderstrand\photos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58D4050A-438A-4C1D-9A73-E55DA932A035}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA3298BF-645B-4168-934C-5B4EF884A1FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,14 +16,14 @@
     <sheet name="PDF Files" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'PDF Files'!$A$1:$E$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'PDF Files'!$A$1:$E$42</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="87">
   <si>
     <t>Year</t>
   </si>
@@ -278,6 +278,12 @@
   </si>
   <si>
     <t>2023-11-18 ezra_ashers_1st_birthday.pdf</t>
+  </si>
+  <si>
+    <t>2025-08-03 Photos at 2500 Pickwick Road</t>
+  </si>
+  <si>
+    <t>2025-08-03_photos_2500_pickwick.pdf</t>
   </si>
 </sst>
 </file>
@@ -634,7 +640,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="3" width="10" customWidth="1"/>
@@ -1228,13 +1234,13 @@
         <v>8</v>
       </c>
       <c r="C35" s="2">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="D35" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="E35" t="s">
-        <v>34</v>
+        <v>86</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.35">
@@ -1242,16 +1248,16 @@
         <v>2025</v>
       </c>
       <c r="B36" s="2">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C36" s="2">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="D36" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E36" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.35">
@@ -1259,16 +1265,16 @@
         <v>2025</v>
       </c>
       <c r="B37" s="2">
+        <v>10</v>
+      </c>
+      <c r="C37" s="2">
         <v>11</v>
       </c>
-      <c r="C37" s="2">
-        <v>22</v>
-      </c>
       <c r="D37" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E37" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.35">
@@ -1279,13 +1285,13 @@
         <v>11</v>
       </c>
       <c r="C38" s="2">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="D38" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E38" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.35">
@@ -1293,33 +1299,33 @@
         <v>2025</v>
       </c>
       <c r="B39" s="2">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C39" s="2">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="D39" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="E39" t="s">
-        <v>81</v>
+        <v>35</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="2">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B40" s="2">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="C40" s="2">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D40" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E40" t="s">
-        <v>37</v>
+        <v>81</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.35">
@@ -1327,22 +1333,39 @@
         <v>2026</v>
       </c>
       <c r="B41" s="2">
+        <v>5</v>
+      </c>
+      <c r="C41" s="2">
+        <v>11</v>
+      </c>
+      <c r="D41" t="s">
+        <v>79</v>
+      </c>
+      <c r="E41" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A42" s="2">
+        <v>2026</v>
+      </c>
+      <c r="B42" s="2">
         <v>6</v>
       </c>
-      <c r="C41" s="2">
+      <c r="C42" s="2">
         <v>24</v>
       </c>
-      <c r="D41" t="s">
+      <c r="D42" t="s">
         <v>83</v>
       </c>
-      <c r="E41" t="s">
+      <c r="E42" t="s">
         <v>38</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E41" xr:uid="{00000000-0009-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E41">
-      <sortCondition ref="D2:D41"/>
+  <autoFilter ref="A1:E42" xr:uid="{00000000-0009-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E42">
+      <sortCondition ref="D2:D42"/>
     </sortState>
   </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>